<commit_message>
Generic template: drop the totals/key-figures block
Keep only the line table (ID, Product, Quantity, Unit Price, per-line
Total, Description). Subtotals and taxes are handled by Odoo, so the
generic bundled template needs no aggregated figures block.
</commit_message>
<xml_diff>
--- a/kalkulations_sync/static/templates/kalkulation_template.xlsx
+++ b/kalkulations_sync/static/templates/kalkulation_template.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -88,12 +88,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -461,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -566,17 +560,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Total (net):</t>
-        </is>
-      </c>
-      <c r="E8" s="8">
-        <f>SUM(E7:E7)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>